<commit_message>
Supplementary ASD-by-CNV figure, Tables S7-S8 and PGS sensitivity
32_supp_asd_by_cnv.R: height, head circumference and BMI by autism
diagnosis within each CNV group (per locus, pooled overgrowth and
undergrowth, SSC probands vs siblings), age- and sex-adjusted, with a
sensitivity analysis adding childhood obesity, adult BMI, height and
autism PGS. Table S7 lists the figure statistics, Table S8 the PGS-adjusted
contrasts. Report (sections 2.8, 3.7), legends, README and handoff updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/manuscript_materials_2026-10-24/supplementary_tables/supp_tables_bmi_effects.xlsx
+++ b/manuscript_materials_2026-10-24/supplementary_tables/supp_tables_bmi_effects.xlsx
@@ -15,12 +15,14 @@
     <sheet name="S5 PGS adjusted" sheetId="23" state="visible" r:id="rId7"/>
     <sheet name="S6 interaction power" sheetId="24" state="visible" r:id="rId8"/>
     <sheet name="notes" sheetId="25" state="visible" r:id="rId9"/>
+    <sheet name="S7 ASD by CNV" sheetId="26" state="visible" r:id="rId10"/>
+    <sheet name="S8 ASD by CNV PGS adj" sheetId="27" state="visible" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3192" uniqueCount="3192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3210" uniqueCount="3210">
   <si>
     <t xml:space="preserve">Trait</t>
   </si>
@@ -9596,6 +9598,60 @@
   </si>
   <si>
     <t xml:space="preserve">Table S6: power to detect modifier x BMI interactions within carriers. For each modifier (sex; each PGS as a continuous z-score) the interaction term BMI x modifier was fitted in GAM y ~ s(age) + BMI * modifier [+ locus]. Power (normal approximation from the term's SE) is given for an interaction as large as the carriers' own BMI effect on that trait, i.e. the BMI effect disappearing in one sex or changing by its full size per SD of PGS; 'detectable interaction' is the smallest effect detectable with 80% power (2.8 x SE). Observed interaction estimates and p-values are listed for completeness.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_noasd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_asd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mean_noasd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">se_noasd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mean_asd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">se_asd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">age_med_noasd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">age_med_asd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">delta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">se</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-carriers (SSC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BMI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">age + sex (same individuals)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S7 ASD by CNV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASD effect (delta, SD; se; p) on height, head circumference and BMI Z within each CNV group, pooled groups and SSC probands vs siblings; GAM y ~ ASD + s(age) + sex [+ cohort + locus]; n_noasd / n_asd; 32_supp_asd_by_cnv.R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S8 ASD by CNV PGS adj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same contrasts in individuals with all four PGS (G2MH carriers, SSC non-carriers), model = covariates added to age + sex; same individuals in every row of a group; 32_supp_asd_by_cnv.R</t>
   </si>
 </sst>
 </file>
@@ -11405,6 +11461,4232 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>363</v>
+      </c>
+      <c r="B1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3192</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3193</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3194</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3195</v>
+      </c>
+      <c r="G1" t="s">
+        <v>3196</v>
+      </c>
+      <c r="H1" t="s">
+        <v>3197</v>
+      </c>
+      <c r="I1" t="s">
+        <v>3198</v>
+      </c>
+      <c r="J1" t="s">
+        <v>3199</v>
+      </c>
+      <c r="K1" t="s">
+        <v>3200</v>
+      </c>
+      <c r="L1" t="s">
+        <v>3201</v>
+      </c>
+      <c r="M1" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="n">
+        <v>149</v>
+      </c>
+      <c r="D2" t="n">
+        <v>80</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.0251257937800607</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.120559141745972</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.364293884869571</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.158089866197612</v>
+      </c>
+      <c r="I2" t="n">
+        <v>12</v>
+      </c>
+      <c r="J2" t="n">
+        <v>12</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.14196725191125</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.2098536591834</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.499435037543136</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" t="n">
+        <v>101</v>
+      </c>
+      <c r="D3" t="n">
+        <v>50</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.243127442568159</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.124013310522639</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.165102707086638</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.191782821285925</v>
+      </c>
+      <c r="I3" t="n">
+        <v>15</v>
+      </c>
+      <c r="J3" t="n">
+        <v>10.5833333333333</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.259114791593682</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.2544158226521</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.310163552951413</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" t="n">
+        <v>213</v>
+      </c>
+      <c r="D4" t="n">
+        <v>65</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-0.520891532177542</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0837772519097082</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-0.460471369393784</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.148298111671817</v>
+      </c>
+      <c r="I4" t="n">
+        <v>14</v>
+      </c>
+      <c r="J4" t="n">
+        <v>11</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.080658206199624</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.178947459600749</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.652537029649672</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" t="n">
+        <v>80</v>
+      </c>
+      <c r="D5" t="n">
+        <v>26</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.0447936302326378</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.117506651130261</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.756214400617207</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.25742424561029</v>
+      </c>
+      <c r="I5" t="n">
+        <v>31</v>
+      </c>
+      <c r="J5" t="n">
+        <v>12</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.303607678948818</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.295692220751988</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.307012860582375</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" t="n">
+        <v>229</v>
+      </c>
+      <c r="D6" t="n">
+        <v>106</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.0319966536761575</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.0883768846005435</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.460425332128425</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.135397250201285</v>
+      </c>
+      <c r="I6" t="n">
+        <v>13</v>
+      </c>
+      <c r="J6" t="n">
+        <v>12</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.185835284094251</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.170539644251403</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.276662905839719</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>91</v>
+      </c>
+      <c r="C7" t="n">
+        <v>314</v>
+      </c>
+      <c r="D7" t="n">
+        <v>115</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-0.275140205905836</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.0721949520441463</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-0.188482640489253</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.121225743892263</v>
+      </c>
+      <c r="I7" t="n">
+        <v>14</v>
+      </c>
+      <c r="J7" t="n">
+        <v>11</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.0810627371915812</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.146273206913886</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.579744993068074</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1596</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2074</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.357536955914081</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.0290327335226672</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.349907393396948</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.0252645362315137</v>
+      </c>
+      <c r="I8" t="n">
+        <v>9.16666666666667</v>
+      </c>
+      <c r="J8" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="K8" t="n">
+        <v>-0.0762824009263388</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.0426443349467162</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.0737288172283092</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="n">
+        <v>129</v>
+      </c>
+      <c r="D9" t="n">
+        <v>72</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.346538640546673</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.124471683270558</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.880598966972302</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.176091118360859</v>
+      </c>
+      <c r="I9" t="n">
+        <v>10.3333333333333</v>
+      </c>
+      <c r="J9" t="n">
+        <v>11.2083333333333</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.405230458888124</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.225435082338719</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.0738179434189932</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="n">
+        <v>77</v>
+      </c>
+      <c r="D10" t="n">
+        <v>43</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-1.13036875033999</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.151693250461725</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-1.58812065965787</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.15259471668149</v>
+      </c>
+      <c r="I10" t="n">
+        <v>15</v>
+      </c>
+      <c r="J10" t="n">
+        <v>10</v>
+      </c>
+      <c r="K10" t="n">
+        <v>-0.124264147155438</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.275278389727191</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.652563979410879</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>116</v>
+      </c>
+      <c r="B11" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" t="n">
+        <v>138</v>
+      </c>
+      <c r="D11" t="n">
+        <v>44</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-0.602956194117033</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.123834484841486</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-0.592410231050582</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.178338704689915</v>
+      </c>
+      <c r="I11" t="n">
+        <v>13</v>
+      </c>
+      <c r="J11" t="n">
+        <v>11</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.0612973356366318</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.246734215778001</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.804086620972098</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" t="n">
+        <v>59</v>
+      </c>
+      <c r="D12" t="n">
+        <v>24</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-0.216461325648302</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.173788781338301</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.275700519818063</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.340589596440618</v>
+      </c>
+      <c r="I12" t="n">
+        <v>16</v>
+      </c>
+      <c r="J12" t="n">
+        <v>12</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.589092252062684</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.415512116084854</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.160371355279043</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>116</v>
+      </c>
+      <c r="B13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" t="n">
+        <v>188</v>
+      </c>
+      <c r="D13" t="n">
+        <v>96</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.169852480942931</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.102867217642005</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.729374355183743</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.158505996407223</v>
+      </c>
+      <c r="I13" t="n">
+        <v>11.4583333333334</v>
+      </c>
+      <c r="J13" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.446721273948788</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.194411418362541</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.0223264695390572</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>116</v>
+      </c>
+      <c r="B14" t="s">
+        <v>91</v>
+      </c>
+      <c r="C14" t="n">
+        <v>215</v>
+      </c>
+      <c r="D14" t="n">
+        <v>87</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-0.791843481694556</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.09760558118579</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-1.0845429716266</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.128626704629971</v>
+      </c>
+      <c r="I14" t="n">
+        <v>13</v>
+      </c>
+      <c r="J14" t="n">
+        <v>10</v>
+      </c>
+      <c r="K14" t="n">
+        <v>-0.0470238418271421</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.183085175517534</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.797481572451074</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>116</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1589</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2060</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-0.103923504281988</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.0312187264679499</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-0.0399234476612568</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.0274324460172736</v>
+      </c>
+      <c r="I15" t="n">
+        <v>9.16666666666667</v>
+      </c>
+      <c r="J15" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.143860522662745</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.0449033453467133</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.0013680411472822</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" t="n">
+        <v>149</v>
+      </c>
+      <c r="D16" t="n">
+        <v>80</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1.38996329378623</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.118963393331665</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1.51072611210404</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.191699212701831</v>
+      </c>
+      <c r="I16" t="n">
+        <v>12</v>
+      </c>
+      <c r="J16" t="n">
+        <v>12</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.123033817250365</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.229890509298447</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.593062117309943</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" t="n">
+        <v>101</v>
+      </c>
+      <c r="D17" t="n">
+        <v>50</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-0.164271816455605</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.133897260397604</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-0.0559295207258598</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.194081715432945</v>
+      </c>
+      <c r="I17" t="n">
+        <v>15</v>
+      </c>
+      <c r="J17" t="n">
+        <v>10.5833333333333</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.107632245594463</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.288260175762136</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.709410464060197</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B18" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" t="n">
+        <v>213</v>
+      </c>
+      <c r="D18" t="n">
+        <v>65</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.372922821512534</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.0954791011387411</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.589625598742078</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.172648850630631</v>
+      </c>
+      <c r="I18" t="n">
+        <v>14</v>
+      </c>
+      <c r="J18" t="n">
+        <v>11</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.164674289484052</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.207255380608476</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.427566807490459</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B19" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" t="n">
+        <v>80</v>
+      </c>
+      <c r="D19" t="n">
+        <v>26</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.617155298104406</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.144312772956587</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.583045329834096</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.305568018624024</v>
+      </c>
+      <c r="I19" t="n">
+        <v>31</v>
+      </c>
+      <c r="J19" t="n">
+        <v>12</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.104549105872159</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.381259692122945</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.784481076715212</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B20" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" t="n">
+        <v>229</v>
+      </c>
+      <c r="D20" t="n">
+        <v>106</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1.1199867014083</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.095360372962775</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1.28318176928311</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.166845323112888</v>
+      </c>
+      <c r="I20" t="n">
+        <v>13</v>
+      </c>
+      <c r="J20" t="n">
+        <v>12</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.078717733211721</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.194602509670464</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.686107561436489</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B21" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" t="n">
+        <v>314</v>
+      </c>
+      <c r="D21" t="n">
+        <v>115</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.200130915669279</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.0789436130084585</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.308949459842975</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.131894339845847</v>
+      </c>
+      <c r="I21" t="n">
+        <v>14</v>
+      </c>
+      <c r="J21" t="n">
+        <v>11</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.151917282383007</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0.166756830741314</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.362810968624776</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B22" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1596</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2074</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.568170416632241</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.0320274985356982</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.677641091751988</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.0297364099908029</v>
+      </c>
+      <c r="I22" t="n">
+        <v>9.16666666666667</v>
+      </c>
+      <c r="J22" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.105398733936998</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0.0490298723630288</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.0316454926010884</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>363</v>
+      </c>
+      <c r="B1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3204</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3192</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3193</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3200</v>
+      </c>
+      <c r="G1" t="s">
+        <v>3201</v>
+      </c>
+      <c r="H1" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D2" t="n">
+        <v>62</v>
+      </c>
+      <c r="E2" t="n">
+        <v>53</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.246408830097647</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.287437948348769</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.393212061676331</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D3" t="n">
+        <v>62</v>
+      </c>
+      <c r="E3" t="n">
+        <v>53</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.249562565242015</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.289201311247452</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.390112197773421</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D4" t="n">
+        <v>62</v>
+      </c>
+      <c r="E4" t="n">
+        <v>53</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.283799735101696</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.284789890396635</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.321261999403464</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D5" t="n">
+        <v>62</v>
+      </c>
+      <c r="E5" t="n">
+        <v>53</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.248750569041655</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.286039276214332</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.386454815785658</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D6" t="n">
+        <v>62</v>
+      </c>
+      <c r="E6" t="n">
+        <v>53</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.213792914610147</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.288725888749372</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.460646442011928</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D7" t="n">
+        <v>62</v>
+      </c>
+      <c r="E7" t="n">
+        <v>53</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.27303418510048</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.286380584451733</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.342610106807432</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D8" t="n">
+        <v>32</v>
+      </c>
+      <c r="E8" t="n">
+        <v>33</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-0.0103887311642216</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.366394446868305</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.977475541031247</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D9" t="n">
+        <v>32</v>
+      </c>
+      <c r="E9" t="n">
+        <v>33</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-0.00755894650122184</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.370439282291789</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.983790046296698</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D10" t="n">
+        <v>32</v>
+      </c>
+      <c r="E10" t="n">
+        <v>33</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-0.00705365474642069</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.370295197983506</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.98486760751988</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D11" t="n">
+        <v>32</v>
+      </c>
+      <c r="E11" t="n">
+        <v>33</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-0.257930325261288</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.325841711792419</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.431830113864931</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D12" t="n">
+        <v>32</v>
+      </c>
+      <c r="E12" t="n">
+        <v>33</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-0.0353314223169525</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.366267161510521</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.923484988337874</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D13" t="n">
+        <v>32</v>
+      </c>
+      <c r="E13" t="n">
+        <v>33</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-0.260108030864657</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.32474672171216</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.426603379352576</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D14" t="n">
+        <v>190</v>
+      </c>
+      <c r="E14" t="n">
+        <v>57</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.0787050378253962</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.193989602119847</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.685308431040914</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D15" t="n">
+        <v>190</v>
+      </c>
+      <c r="E15" t="n">
+        <v>57</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.0810487781376669</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.193489955734377</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.675678022478089</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D16" t="n">
+        <v>190</v>
+      </c>
+      <c r="E16" t="n">
+        <v>57</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.0705590284467247</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.193330232970064</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.715456600409545</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D17" t="n">
+        <v>190</v>
+      </c>
+      <c r="E17" t="n">
+        <v>57</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-0.00326108659631222</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.171764304678004</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.984868124254395</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D18" t="n">
+        <v>190</v>
+      </c>
+      <c r="E18" t="n">
+        <v>57</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.061042553264989</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.195625587092602</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.755281687445595</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" t="s">
+        <v>54</v>
+      </c>
+      <c r="C19" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D19" t="n">
+        <v>190</v>
+      </c>
+      <c r="E19" t="n">
+        <v>57</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-0.0082688475999379</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.172588982366745</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.961827643628967</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" t="s">
+        <v>67</v>
+      </c>
+      <c r="C20" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D20" t="n">
+        <v>70</v>
+      </c>
+      <c r="E20" t="n">
+        <v>24</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.0552941707737382</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.330741188715454</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.86761178809641</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" t="s">
+        <v>67</v>
+      </c>
+      <c r="C21" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D21" t="n">
+        <v>70</v>
+      </c>
+      <c r="E21" t="n">
+        <v>24</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.116576909224686</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.321665414663391</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.717924203767946</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22" t="s">
+        <v>67</v>
+      </c>
+      <c r="C22" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D22" t="n">
+        <v>70</v>
+      </c>
+      <c r="E22" t="n">
+        <v>24</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.0738213734174935</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.329369457690398</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.823184332295808</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D23" t="n">
+        <v>70</v>
+      </c>
+      <c r="E23" t="n">
+        <v>24</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-0.00113658024060909</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.290650565868434</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.996889014709591</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B24" t="s">
+        <v>67</v>
+      </c>
+      <c r="C24" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D24" t="n">
+        <v>70</v>
+      </c>
+      <c r="E24" t="n">
+        <v>24</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.0737033679099923</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.334215875929956</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.825980367051412</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" t="s">
+        <v>67</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D25" t="n">
+        <v>70</v>
+      </c>
+      <c r="E25" t="n">
+        <v>24</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.0726249035029007</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.280234306553721</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.796159619586805</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B26" t="s">
+        <v>79</v>
+      </c>
+      <c r="C26" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D26" t="n">
+        <v>132</v>
+      </c>
+      <c r="E26" t="n">
+        <v>77</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.215892276455653</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.210718373191184</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.306813287082652</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D27" t="n">
+        <v>132</v>
+      </c>
+      <c r="E27" t="n">
+        <v>77</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.212890495311038</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.210507819402857</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.313094455079557</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D28" t="n">
+        <v>132</v>
+      </c>
+      <c r="E28" t="n">
+        <v>77</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.243661484977736</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.208463033876474</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.243866719260595</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>14</v>
+      </c>
+      <c r="B29" t="s">
+        <v>79</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D29" t="n">
+        <v>132</v>
+      </c>
+      <c r="E29" t="n">
+        <v>77</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.192916297638787</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.20187536435011</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.340425258591986</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30" t="s">
+        <v>79</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D30" t="n">
+        <v>132</v>
+      </c>
+      <c r="E30" t="n">
+        <v>77</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.208327337492605</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.211786758245841</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.326476038007141</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>14</v>
+      </c>
+      <c r="B31" t="s">
+        <v>79</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D31" t="n">
+        <v>132</v>
+      </c>
+      <c r="E31" t="n">
+        <v>77</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.211497929578147</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.200756729062957</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.293410484937051</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>14</v>
+      </c>
+      <c r="B32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C32" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D32" t="n">
+        <v>222</v>
+      </c>
+      <c r="E32" t="n">
+        <v>90</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.00229891760647268</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.171028100612922</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.989284143347377</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B33" t="s">
+        <v>91</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D33" t="n">
+        <v>222</v>
+      </c>
+      <c r="E33" t="n">
+        <v>90</v>
+      </c>
+      <c r="F33" t="n">
+        <v>-0.000740393035097341</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.171035969226496</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.996548908911</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>14</v>
+      </c>
+      <c r="B34" t="s">
+        <v>91</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D34" t="n">
+        <v>222</v>
+      </c>
+      <c r="E34" t="n">
+        <v>90</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-0.0046331880452741</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.17070169374964</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.978364272043241</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>14</v>
+      </c>
+      <c r="B35" t="s">
+        <v>91</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D35" t="n">
+        <v>222</v>
+      </c>
+      <c r="E35" t="n">
+        <v>90</v>
+      </c>
+      <c r="F35" t="n">
+        <v>-0.107361934037335</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.150768657332888</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.476950738499955</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>14</v>
+      </c>
+      <c r="B36" t="s">
+        <v>91</v>
+      </c>
+      <c r="C36" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D36" t="n">
+        <v>222</v>
+      </c>
+      <c r="E36" t="n">
+        <v>90</v>
+      </c>
+      <c r="F36" t="n">
+        <v>-0.0179499842947393</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.171933914187896</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.916920381213254</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>14</v>
+      </c>
+      <c r="B37" t="s">
+        <v>91</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D37" t="n">
+        <v>222</v>
+      </c>
+      <c r="E37" t="n">
+        <v>90</v>
+      </c>
+      <c r="F37" t="n">
+        <v>-0.123745810020017</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.151703517431286</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.41531203431258</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>14</v>
+      </c>
+      <c r="B38" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C38" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1438</v>
+      </c>
+      <c r="E38" t="n">
+        <v>1895</v>
+      </c>
+      <c r="F38" t="n">
+        <v>-0.0853468717051047</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.0446379522884787</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.0559645767964572</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>14</v>
+      </c>
+      <c r="B39" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D39" t="n">
+        <v>1438</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1895</v>
+      </c>
+      <c r="F39" t="n">
+        <v>-0.0875078688786038</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.0445234545424081</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.0494472369703637</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>14</v>
+      </c>
+      <c r="B40" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C40" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1438</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1895</v>
+      </c>
+      <c r="F40" t="n">
+        <v>-0.0890643044552751</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.0444429861719346</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.0451496684919105</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>14</v>
+      </c>
+      <c r="B41" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D41" t="n">
+        <v>1438</v>
+      </c>
+      <c r="E41" t="n">
+        <v>1895</v>
+      </c>
+      <c r="F41" t="n">
+        <v>-0.12758114976672</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.0400685377958677</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.0014655948073015</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>14</v>
+      </c>
+      <c r="B42" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C42" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1438</v>
+      </c>
+      <c r="E42" t="n">
+        <v>1895</v>
+      </c>
+      <c r="F42" t="n">
+        <v>-0.101714411665522</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.0451947191189705</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.0244771164885874</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>14</v>
+      </c>
+      <c r="B43" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C43" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D43" t="n">
+        <v>1438</v>
+      </c>
+      <c r="E43" t="n">
+        <v>1895</v>
+      </c>
+      <c r="F43" t="n">
+        <v>-0.144246405761281</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.0402230032544637</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.00034040691459564</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>116</v>
+      </c>
+      <c r="B44" t="s">
+        <v>24</v>
+      </c>
+      <c r="C44" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D44" t="n">
+        <v>52</v>
+      </c>
+      <c r="E44" t="n">
+        <v>46</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.328013016722698</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.325818661094506</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.316714939805653</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>116</v>
+      </c>
+      <c r="B45" t="s">
+        <v>24</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D45" t="n">
+        <v>52</v>
+      </c>
+      <c r="E45" t="n">
+        <v>46</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.31577812030197</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.324972584241236</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.333777396517041</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>116</v>
+      </c>
+      <c r="B46" t="s">
+        <v>24</v>
+      </c>
+      <c r="C46" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D46" t="n">
+        <v>52</v>
+      </c>
+      <c r="E46" t="n">
+        <v>46</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.408625911486194</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.322901775419248</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.208934439070607</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>116</v>
+      </c>
+      <c r="B47" t="s">
+        <v>24</v>
+      </c>
+      <c r="C47" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D47" t="n">
+        <v>52</v>
+      </c>
+      <c r="E47" t="n">
+        <v>46</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.328169925819663</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.327580219592803</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.319108245627093</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>116</v>
+      </c>
+      <c r="B48" t="s">
+        <v>24</v>
+      </c>
+      <c r="C48" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D48" t="n">
+        <v>52</v>
+      </c>
+      <c r="E48" t="n">
+        <v>46</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.318090725667693</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.330948586428559</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0.339036105478578</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>116</v>
+      </c>
+      <c r="B49" t="s">
+        <v>24</v>
+      </c>
+      <c r="C49" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D49" t="n">
+        <v>52</v>
+      </c>
+      <c r="E49" t="n">
+        <v>46</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.37195557834225</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.332731948342733</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0.26665987096148</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>116</v>
+      </c>
+      <c r="B50" t="s">
+        <v>40</v>
+      </c>
+      <c r="C50" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D50" t="n">
+        <v>24</v>
+      </c>
+      <c r="E50" t="n">
+        <v>29</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.0946240311488799</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0.3824474212724</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0.805663115956914</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>116</v>
+      </c>
+      <c r="B51" t="s">
+        <v>40</v>
+      </c>
+      <c r="C51" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D51" t="n">
+        <v>24</v>
+      </c>
+      <c r="E51" t="n">
+        <v>29</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.0984929044685381</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.384254489706453</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0.798845058506272</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>116</v>
+      </c>
+      <c r="B52" t="s">
+        <v>40</v>
+      </c>
+      <c r="C52" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D52" t="n">
+        <v>24</v>
+      </c>
+      <c r="E52" t="n">
+        <v>29</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.0936178231687692</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0.386847400271189</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0.809854329238885</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>116</v>
+      </c>
+      <c r="B53" t="s">
+        <v>40</v>
+      </c>
+      <c r="C53" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D53" t="n">
+        <v>24</v>
+      </c>
+      <c r="E53" t="n">
+        <v>29</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.144445512952939</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0.390541152871609</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0.713184307985075</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>116</v>
+      </c>
+      <c r="B54" t="s">
+        <v>40</v>
+      </c>
+      <c r="C54" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D54" t="n">
+        <v>24</v>
+      </c>
+      <c r="E54" t="n">
+        <v>29</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.0974155805591745</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0.38676863804467</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0.802263170150186</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>116</v>
+      </c>
+      <c r="B55" t="s">
+        <v>40</v>
+      </c>
+      <c r="C55" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D55" t="n">
+        <v>24</v>
+      </c>
+      <c r="E55" t="n">
+        <v>29</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.155434731794341</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0.400693737847706</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0.699993413844192</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>116</v>
+      </c>
+      <c r="B56" t="s">
+        <v>54</v>
+      </c>
+      <c r="C56" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D56" t="n">
+        <v>123</v>
+      </c>
+      <c r="E56" t="n">
+        <v>38</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.11959828026495</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0.265683264430133</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0.653227564790817</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>116</v>
+      </c>
+      <c r="B57" t="s">
+        <v>54</v>
+      </c>
+      <c r="C57" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D57" t="n">
+        <v>123</v>
+      </c>
+      <c r="E57" t="n">
+        <v>38</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.1420081621782</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0.264651339825084</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0.592326605012739</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>116</v>
+      </c>
+      <c r="B58" t="s">
+        <v>54</v>
+      </c>
+      <c r="C58" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D58" t="n">
+        <v>123</v>
+      </c>
+      <c r="E58" t="n">
+        <v>38</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.152028019318361</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0.265369389191835</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0.567551790708012</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>116</v>
+      </c>
+      <c r="B59" t="s">
+        <v>54</v>
+      </c>
+      <c r="C59" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D59" t="n">
+        <v>123</v>
+      </c>
+      <c r="E59" t="n">
+        <v>38</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.109329340910517</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0.266127649580501</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0.681777523792403</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>116</v>
+      </c>
+      <c r="B60" t="s">
+        <v>54</v>
+      </c>
+      <c r="C60" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D60" t="n">
+        <v>123</v>
+      </c>
+      <c r="E60" t="n">
+        <v>38</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.0685303432635156</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0.266525574254201</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0.797424988123241</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>116</v>
+      </c>
+      <c r="B61" t="s">
+        <v>54</v>
+      </c>
+      <c r="C61" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D61" t="n">
+        <v>123</v>
+      </c>
+      <c r="E61" t="n">
+        <v>38</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.110564744262294</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0.267162978338893</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0.679571242645953</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>116</v>
+      </c>
+      <c r="B62" t="s">
+        <v>67</v>
+      </c>
+      <c r="C62" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D62" t="n">
+        <v>49</v>
+      </c>
+      <c r="E62" t="n">
+        <v>22</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.0563522777688231</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0.459408334896264</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0.902760739626356</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>116</v>
+      </c>
+      <c r="B63" t="s">
+        <v>67</v>
+      </c>
+      <c r="C63" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D63" t="n">
+        <v>49</v>
+      </c>
+      <c r="E63" t="n">
+        <v>22</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.122683853996711</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0.460444281574653</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0.790767654707887</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>116</v>
+      </c>
+      <c r="B64" t="s">
+        <v>67</v>
+      </c>
+      <c r="C64" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D64" t="n">
+        <v>49</v>
+      </c>
+      <c r="E64" t="n">
+        <v>22</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0.081934072720455</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0.458829614363471</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0.858849072579508</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>116</v>
+      </c>
+      <c r="B65" t="s">
+        <v>67</v>
+      </c>
+      <c r="C65" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D65" t="n">
+        <v>49</v>
+      </c>
+      <c r="E65" t="n">
+        <v>22</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0.0721291316885911</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0.441539813564817</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0.870758775314025</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>116</v>
+      </c>
+      <c r="B66" t="s">
+        <v>67</v>
+      </c>
+      <c r="C66" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D66" t="n">
+        <v>49</v>
+      </c>
+      <c r="E66" t="n">
+        <v>22</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0.060431178912559</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0.466930894538523</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0.897438258557441</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>116</v>
+      </c>
+      <c r="B67" t="s">
+        <v>67</v>
+      </c>
+      <c r="C67" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D67" t="n">
+        <v>49</v>
+      </c>
+      <c r="E67" t="n">
+        <v>22</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0.149891197748564</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0.44611721879836</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0.738044188608745</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>116</v>
+      </c>
+      <c r="B68" t="s">
+        <v>79</v>
+      </c>
+      <c r="C68" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D68" t="n">
+        <v>101</v>
+      </c>
+      <c r="E68" t="n">
+        <v>68</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0.328374723725307</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0.255993364214743</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0.201428341828561</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>116</v>
+      </c>
+      <c r="B69" t="s">
+        <v>79</v>
+      </c>
+      <c r="C69" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D69" t="n">
+        <v>101</v>
+      </c>
+      <c r="E69" t="n">
+        <v>68</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0.328506075641838</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0.253846002304323</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0.197492285584251</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>116</v>
+      </c>
+      <c r="B70" t="s">
+        <v>79</v>
+      </c>
+      <c r="C70" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D70" t="n">
+        <v>101</v>
+      </c>
+      <c r="E70" t="n">
+        <v>68</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0.382483189571958</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0.253318392637567</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0.133045292966875</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>116</v>
+      </c>
+      <c r="B71" t="s">
+        <v>79</v>
+      </c>
+      <c r="C71" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D71" t="n">
+        <v>101</v>
+      </c>
+      <c r="E71" t="n">
+        <v>68</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0.308830930200847</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0.254352552707095</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0.226468774586861</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>116</v>
+      </c>
+      <c r="B72" t="s">
+        <v>79</v>
+      </c>
+      <c r="C72" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D72" t="n">
+        <v>101</v>
+      </c>
+      <c r="E72" t="n">
+        <v>68</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0.337337400878247</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0.258604508376669</v>
+      </c>
+      <c r="H72" t="n">
+        <v>0.193956464209481</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>116</v>
+      </c>
+      <c r="B73" t="s">
+        <v>79</v>
+      </c>
+      <c r="C73" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D73" t="n">
+        <v>101</v>
+      </c>
+      <c r="E73" t="n">
+        <v>68</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0.358578799765719</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0.253621470383373</v>
+      </c>
+      <c r="H73" t="n">
+        <v>0.159389196300167</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s">
+        <v>116</v>
+      </c>
+      <c r="B74" t="s">
+        <v>91</v>
+      </c>
+      <c r="C74" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D74" t="n">
+        <v>147</v>
+      </c>
+      <c r="E74" t="n">
+        <v>67</v>
+      </c>
+      <c r="F74" t="n">
+        <v>0.0264711123962536</v>
+      </c>
+      <c r="G74" t="n">
+        <v>0.219307119767775</v>
+      </c>
+      <c r="H74" t="n">
+        <v>0.904043310738098</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="s">
+        <v>116</v>
+      </c>
+      <c r="B75" t="s">
+        <v>91</v>
+      </c>
+      <c r="C75" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D75" t="n">
+        <v>147</v>
+      </c>
+      <c r="E75" t="n">
+        <v>67</v>
+      </c>
+      <c r="F75" t="n">
+        <v>0.0417600545387198</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0.218510510958152</v>
+      </c>
+      <c r="H75" t="n">
+        <v>0.84862613939432</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="s">
+        <v>116</v>
+      </c>
+      <c r="B76" t="s">
+        <v>91</v>
+      </c>
+      <c r="C76" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D76" t="n">
+        <v>147</v>
+      </c>
+      <c r="E76" t="n">
+        <v>67</v>
+      </c>
+      <c r="F76" t="n">
+        <v>0.0400367875491041</v>
+      </c>
+      <c r="G76" t="n">
+        <v>0.219462048026712</v>
+      </c>
+      <c r="H76" t="n">
+        <v>0.855423888552443</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="s">
+        <v>116</v>
+      </c>
+      <c r="B77" t="s">
+        <v>91</v>
+      </c>
+      <c r="C77" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D77" t="n">
+        <v>147</v>
+      </c>
+      <c r="E77" t="n">
+        <v>67</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0.0167486166213365</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0.220049390292408</v>
+      </c>
+      <c r="H77" t="n">
+        <v>0.939403214779819</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s">
+        <v>116</v>
+      </c>
+      <c r="B78" t="s">
+        <v>91</v>
+      </c>
+      <c r="C78" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D78" t="n">
+        <v>147</v>
+      </c>
+      <c r="E78" t="n">
+        <v>67</v>
+      </c>
+      <c r="F78" t="n">
+        <v>-0.00131932472863355</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0.219889510070034</v>
+      </c>
+      <c r="H78" t="n">
+        <v>0.995218580843222</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s">
+        <v>116</v>
+      </c>
+      <c r="B79" t="s">
+        <v>91</v>
+      </c>
+      <c r="C79" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D79" t="n">
+        <v>147</v>
+      </c>
+      <c r="E79" t="n">
+        <v>67</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0.0147573438773111</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0.220509145627298</v>
+      </c>
+      <c r="H79" t="n">
+        <v>0.946708147181502</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s">
+        <v>116</v>
+      </c>
+      <c r="B80" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C80" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D80" t="n">
+        <v>1431</v>
+      </c>
+      <c r="E80" t="n">
+        <v>1882</v>
+      </c>
+      <c r="F80" t="n">
+        <v>0.145391271679616</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0.0468162435299946</v>
+      </c>
+      <c r="H80" t="n">
+        <v>0.00191518210736431</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="s">
+        <v>116</v>
+      </c>
+      <c r="B81" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C81" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D81" t="n">
+        <v>1431</v>
+      </c>
+      <c r="E81" t="n">
+        <v>1882</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0.143287894574785</v>
+      </c>
+      <c r="G81" t="n">
+        <v>0.0467018209124753</v>
+      </c>
+      <c r="H81" t="n">
+        <v>0.00217137406836672</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="s">
+        <v>116</v>
+      </c>
+      <c r="B82" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C82" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D82" t="n">
+        <v>1431</v>
+      </c>
+      <c r="E82" t="n">
+        <v>1882</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0.141241479766543</v>
+      </c>
+      <c r="G82" t="n">
+        <v>0.0465670893376102</v>
+      </c>
+      <c r="H82" t="n">
+        <v>0.00243954787960056</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="s">
+        <v>116</v>
+      </c>
+      <c r="B83" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C83" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D83" t="n">
+        <v>1431</v>
+      </c>
+      <c r="E83" t="n">
+        <v>1882</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0.130694188065302</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0.0464042808820998</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0.00488491680821262</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="s">
+        <v>116</v>
+      </c>
+      <c r="B84" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C84" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D84" t="n">
+        <v>1431</v>
+      </c>
+      <c r="E84" t="n">
+        <v>1882</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0.128376903002713</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0.0473952651692804</v>
+      </c>
+      <c r="H84" t="n">
+        <v>0.00679066433629246</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="s">
+        <v>116</v>
+      </c>
+      <c r="B85" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C85" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D85" t="n">
+        <v>1431</v>
+      </c>
+      <c r="E85" t="n">
+        <v>1882</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0.109315993085145</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0.0466654654057952</v>
+      </c>
+      <c r="H85" t="n">
+        <v>0.0192117121149853</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B86" t="s">
+        <v>24</v>
+      </c>
+      <c r="C86" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D86" t="n">
+        <v>62</v>
+      </c>
+      <c r="E86" t="n">
+        <v>53</v>
+      </c>
+      <c r="F86" t="n">
+        <v>0.142177890522635</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0.321141198173728</v>
+      </c>
+      <c r="H86" t="n">
+        <v>0.658849739032046</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B87" t="s">
+        <v>24</v>
+      </c>
+      <c r="C87" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D87" t="n">
+        <v>62</v>
+      </c>
+      <c r="E87" t="n">
+        <v>53</v>
+      </c>
+      <c r="F87" t="n">
+        <v>0.114027572682659</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0.319623890556269</v>
+      </c>
+      <c r="H87" t="n">
+        <v>0.721976365831889</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B88" t="s">
+        <v>24</v>
+      </c>
+      <c r="C88" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D88" t="n">
+        <v>62</v>
+      </c>
+      <c r="E88" t="n">
+        <v>53</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0.210625729882404</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0.304174956563654</v>
+      </c>
+      <c r="H88" t="n">
+        <v>0.490155405561566</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B89" t="s">
+        <v>24</v>
+      </c>
+      <c r="C89" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D89" t="n">
+        <v>62</v>
+      </c>
+      <c r="E89" t="n">
+        <v>53</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0.133800427275531</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0.321176526690126</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0.677810722890115</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B90" t="s">
+        <v>24</v>
+      </c>
+      <c r="C90" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D90" t="n">
+        <v>62</v>
+      </c>
+      <c r="E90" t="n">
+        <v>53</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0.159376826316846</v>
+      </c>
+      <c r="G90" t="n">
+        <v>0.323818432984445</v>
+      </c>
+      <c r="H90" t="n">
+        <v>0.623602009281967</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B91" t="s">
+        <v>24</v>
+      </c>
+      <c r="C91" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D91" t="n">
+        <v>62</v>
+      </c>
+      <c r="E91" t="n">
+        <v>53</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0.188425526833274</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0.3092242675225</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0.54362209899915</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B92" t="s">
+        <v>40</v>
+      </c>
+      <c r="C92" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D92" t="n">
+        <v>32</v>
+      </c>
+      <c r="E92" t="n">
+        <v>33</v>
+      </c>
+      <c r="F92" t="n">
+        <v>0.45119100454886</v>
+      </c>
+      <c r="G92" t="n">
+        <v>0.395730910149638</v>
+      </c>
+      <c r="H92" t="n">
+        <v>0.258832880090636</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B93" t="s">
+        <v>40</v>
+      </c>
+      <c r="C93" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D93" t="n">
+        <v>32</v>
+      </c>
+      <c r="E93" t="n">
+        <v>33</v>
+      </c>
+      <c r="F93" t="n">
+        <v>0.446575434811426</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0.40004857064194</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0.268895885264267</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B94" t="s">
+        <v>40</v>
+      </c>
+      <c r="C94" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D94" t="n">
+        <v>32</v>
+      </c>
+      <c r="E94" t="n">
+        <v>33</v>
+      </c>
+      <c r="F94" t="n">
+        <v>0.515370463721499</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0.379270780512622</v>
+      </c>
+      <c r="H94" t="n">
+        <v>0.179456580569141</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B95" t="s">
+        <v>40</v>
+      </c>
+      <c r="C95" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D95" t="n">
+        <v>32</v>
+      </c>
+      <c r="E95" t="n">
+        <v>33</v>
+      </c>
+      <c r="F95" t="n">
+        <v>0.396364996389862</v>
+      </c>
+      <c r="G95" t="n">
+        <v>0.403244738329559</v>
+      </c>
+      <c r="H95" t="n">
+        <v>0.329720068706342</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B96" t="s">
+        <v>40</v>
+      </c>
+      <c r="C96" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D96" t="n">
+        <v>32</v>
+      </c>
+      <c r="E96" t="n">
+        <v>33</v>
+      </c>
+      <c r="F96" t="n">
+        <v>0.497515373760926</v>
+      </c>
+      <c r="G96" t="n">
+        <v>0.387093968626683</v>
+      </c>
+      <c r="H96" t="n">
+        <v>0.203810995768832</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B97" t="s">
+        <v>40</v>
+      </c>
+      <c r="C97" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D97" t="n">
+        <v>32</v>
+      </c>
+      <c r="E97" t="n">
+        <v>33</v>
+      </c>
+      <c r="F97" t="n">
+        <v>0.481527733558462</v>
+      </c>
+      <c r="G97" t="n">
+        <v>0.377449210567116</v>
+      </c>
+      <c r="H97" t="n">
+        <v>0.207408588764097</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B98" t="s">
+        <v>54</v>
+      </c>
+      <c r="C98" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D98" t="n">
+        <v>190</v>
+      </c>
+      <c r="E98" t="n">
+        <v>57</v>
+      </c>
+      <c r="F98" t="n">
+        <v>0.290543186753769</v>
+      </c>
+      <c r="G98" t="n">
+        <v>0.22093097909585</v>
+      </c>
+      <c r="H98" t="n">
+        <v>0.189725825308412</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B99" t="s">
+        <v>54</v>
+      </c>
+      <c r="C99" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D99" t="n">
+        <v>190</v>
+      </c>
+      <c r="E99" t="n">
+        <v>57</v>
+      </c>
+      <c r="F99" t="n">
+        <v>0.294596148881966</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0.219000814009636</v>
+      </c>
+      <c r="H99" t="n">
+        <v>0.179830580952468</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B100" t="s">
+        <v>54</v>
+      </c>
+      <c r="C100" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D100" t="n">
+        <v>190</v>
+      </c>
+      <c r="E100" t="n">
+        <v>57</v>
+      </c>
+      <c r="F100" t="n">
+        <v>0.316071701968031</v>
+      </c>
+      <c r="G100" t="n">
+        <v>0.211584370909005</v>
+      </c>
+      <c r="H100" t="n">
+        <v>0.136527378079756</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B101" t="s">
+        <v>54</v>
+      </c>
+      <c r="C101" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D101" t="n">
+        <v>190</v>
+      </c>
+      <c r="E101" t="n">
+        <v>57</v>
+      </c>
+      <c r="F101" t="n">
+        <v>0.300590230751864</v>
+      </c>
+      <c r="G101" t="n">
+        <v>0.221471627168126</v>
+      </c>
+      <c r="H101" t="n">
+        <v>0.17597454036227</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B102" t="s">
+        <v>54</v>
+      </c>
+      <c r="C102" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D102" t="n">
+        <v>190</v>
+      </c>
+      <c r="E102" t="n">
+        <v>57</v>
+      </c>
+      <c r="F102" t="n">
+        <v>0.277881155236881</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0.22294750351626</v>
+      </c>
+      <c r="H102" t="n">
+        <v>0.213828726289493</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B103" t="s">
+        <v>54</v>
+      </c>
+      <c r="C103" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D103" t="n">
+        <v>190</v>
+      </c>
+      <c r="E103" t="n">
+        <v>57</v>
+      </c>
+      <c r="F103" t="n">
+        <v>0.311801591976197</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0.213995605363755</v>
+      </c>
+      <c r="H103" t="n">
+        <v>0.146421575857505</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B104" t="s">
+        <v>67</v>
+      </c>
+      <c r="C104" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D104" t="n">
+        <v>70</v>
+      </c>
+      <c r="E104" t="n">
+        <v>24</v>
+      </c>
+      <c r="F104" t="n">
+        <v>-0.0214752873574504</v>
+      </c>
+      <c r="G104" t="n">
+        <v>0.38626023782329</v>
+      </c>
+      <c r="H104" t="n">
+        <v>0.955788114489277</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B105" t="s">
+        <v>67</v>
+      </c>
+      <c r="C105" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D105" t="n">
+        <v>70</v>
+      </c>
+      <c r="E105" t="n">
+        <v>24</v>
+      </c>
+      <c r="F105" t="n">
+        <v>0.0240785384740499</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0.384101265980327</v>
+      </c>
+      <c r="H105" t="n">
+        <v>0.95015875761822</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B106" t="s">
+        <v>67</v>
+      </c>
+      <c r="C106" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D106" t="n">
+        <v>70</v>
+      </c>
+      <c r="E106" t="n">
+        <v>24</v>
+      </c>
+      <c r="F106" t="n">
+        <v>0.0017842964578811</v>
+      </c>
+      <c r="G106" t="n">
+        <v>0.383369011400121</v>
+      </c>
+      <c r="H106" t="n">
+        <v>0.996297112356287</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B107" t="s">
+        <v>67</v>
+      </c>
+      <c r="C107" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D107" t="n">
+        <v>70</v>
+      </c>
+      <c r="E107" t="n">
+        <v>24</v>
+      </c>
+      <c r="F107" t="n">
+        <v>-0.0210566744648927</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0.388911991313203</v>
+      </c>
+      <c r="H107" t="n">
+        <v>0.95694575430424</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B108" t="s">
+        <v>67</v>
+      </c>
+      <c r="C108" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D108" t="n">
+        <v>70</v>
+      </c>
+      <c r="E108" t="n">
+        <v>24</v>
+      </c>
+      <c r="F108" t="n">
+        <v>0.0277546744828667</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0.387908839827647</v>
+      </c>
+      <c r="H108" t="n">
+        <v>0.943124673610645</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B109" t="s">
+        <v>67</v>
+      </c>
+      <c r="C109" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D109" t="n">
+        <v>70</v>
+      </c>
+      <c r="E109" t="n">
+        <v>24</v>
+      </c>
+      <c r="F109" t="n">
+        <v>0.0717950674688833</v>
+      </c>
+      <c r="G109" t="n">
+        <v>0.38801797961348</v>
+      </c>
+      <c r="H109" t="n">
+        <v>0.853651325863355</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B110" t="s">
+        <v>79</v>
+      </c>
+      <c r="C110" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D110" t="n">
+        <v>132</v>
+      </c>
+      <c r="E110" t="n">
+        <v>77</v>
+      </c>
+      <c r="F110" t="n">
+        <v>0.0675447435435194</v>
+      </c>
+      <c r="G110" t="n">
+        <v>0.238910164441301</v>
+      </c>
+      <c r="H110" t="n">
+        <v>0.777682907968645</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B111" t="s">
+        <v>79</v>
+      </c>
+      <c r="C111" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D111" t="n">
+        <v>132</v>
+      </c>
+      <c r="E111" t="n">
+        <v>77</v>
+      </c>
+      <c r="F111" t="n">
+        <v>0.062563156709571</v>
+      </c>
+      <c r="G111" t="n">
+        <v>0.236547844492005</v>
+      </c>
+      <c r="H111" t="n">
+        <v>0.791679398993708</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B112" t="s">
+        <v>79</v>
+      </c>
+      <c r="C112" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D112" t="n">
+        <v>132</v>
+      </c>
+      <c r="E112" t="n">
+        <v>77</v>
+      </c>
+      <c r="F112" t="n">
+        <v>0.117520744205504</v>
+      </c>
+      <c r="G112" t="n">
+        <v>0.230480455701813</v>
+      </c>
+      <c r="H112" t="n">
+        <v>0.610687904364387</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B113" t="s">
+        <v>79</v>
+      </c>
+      <c r="C113" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D113" t="n">
+        <v>132</v>
+      </c>
+      <c r="E113" t="n">
+        <v>77</v>
+      </c>
+      <c r="F113" t="n">
+        <v>0.0654341605511128</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0.238834415610522</v>
+      </c>
+      <c r="H113" t="n">
+        <v>0.784389341766306</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B114" t="s">
+        <v>79</v>
+      </c>
+      <c r="C114" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D114" t="n">
+        <v>132</v>
+      </c>
+      <c r="E114" t="n">
+        <v>77</v>
+      </c>
+      <c r="F114" t="n">
+        <v>0.088832204789112</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0.239220536219502</v>
+      </c>
+      <c r="H114" t="n">
+        <v>0.71077837384843</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B115" t="s">
+        <v>79</v>
+      </c>
+      <c r="C115" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D115" t="n">
+        <v>132</v>
+      </c>
+      <c r="E115" t="n">
+        <v>77</v>
+      </c>
+      <c r="F115" t="n">
+        <v>0.127575906371971</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0.231613842553308</v>
+      </c>
+      <c r="H115" t="n">
+        <v>0.582386759706422</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B116" t="s">
+        <v>91</v>
+      </c>
+      <c r="C116" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D116" t="n">
+        <v>222</v>
+      </c>
+      <c r="E116" t="n">
+        <v>90</v>
+      </c>
+      <c r="F116" t="n">
+        <v>0.323967839841059</v>
+      </c>
+      <c r="G116" t="n">
+        <v>0.191399254632694</v>
+      </c>
+      <c r="H116" t="n">
+        <v>0.0915473666574875</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B117" t="s">
+        <v>91</v>
+      </c>
+      <c r="C117" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D117" t="n">
+        <v>222</v>
+      </c>
+      <c r="E117" t="n">
+        <v>90</v>
+      </c>
+      <c r="F117" t="n">
+        <v>0.317285984185868</v>
+      </c>
+      <c r="G117" t="n">
+        <v>0.190449718514585</v>
+      </c>
+      <c r="H117" t="n">
+        <v>0.0967468485781615</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B118" t="s">
+        <v>91</v>
+      </c>
+      <c r="C118" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D118" t="n">
+        <v>222</v>
+      </c>
+      <c r="E118" t="n">
+        <v>90</v>
+      </c>
+      <c r="F118" t="n">
+        <v>0.350177334171098</v>
+      </c>
+      <c r="G118" t="n">
+        <v>0.183080797570901</v>
+      </c>
+      <c r="H118" t="n">
+        <v>0.0567268476279486</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B119" t="s">
+        <v>91</v>
+      </c>
+      <c r="C119" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D119" t="n">
+        <v>222</v>
+      </c>
+      <c r="E119" t="n">
+        <v>90</v>
+      </c>
+      <c r="F119" t="n">
+        <v>0.327342853762379</v>
+      </c>
+      <c r="G119" t="n">
+        <v>0.192258172943315</v>
+      </c>
+      <c r="H119" t="n">
+        <v>0.089661141615748</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B120" t="s">
+        <v>91</v>
+      </c>
+      <c r="C120" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D120" t="n">
+        <v>222</v>
+      </c>
+      <c r="E120" t="n">
+        <v>90</v>
+      </c>
+      <c r="F120" t="n">
+        <v>0.334850778107422</v>
+      </c>
+      <c r="G120" t="n">
+        <v>0.192712648031203</v>
+      </c>
+      <c r="H120" t="n">
+        <v>0.0833001903449014</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B121" t="s">
+        <v>91</v>
+      </c>
+      <c r="C121" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D121" t="n">
+        <v>222</v>
+      </c>
+      <c r="E121" t="n">
+        <v>90</v>
+      </c>
+      <c r="F121" t="n">
+        <v>0.351684416161286</v>
+      </c>
+      <c r="G121" t="n">
+        <v>0.18488078248506</v>
+      </c>
+      <c r="H121" t="n">
+        <v>0.0580964081533915</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B122" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C122" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D122" t="n">
+        <v>1438</v>
+      </c>
+      <c r="E122" t="n">
+        <v>1895</v>
+      </c>
+      <c r="F122" t="n">
+        <v>0.12597325966606</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0.0513771406034049</v>
+      </c>
+      <c r="H122" t="n">
+        <v>0.0142601939783087</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B123" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C123" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D123" t="n">
+        <v>1438</v>
+      </c>
+      <c r="E123" t="n">
+        <v>1895</v>
+      </c>
+      <c r="F123" t="n">
+        <v>0.120151922557871</v>
+      </c>
+      <c r="G123" t="n">
+        <v>0.0505635923196123</v>
+      </c>
+      <c r="H123" t="n">
+        <v>0.0175457442368672</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B124" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C124" t="s">
+        <v>1630</v>
+      </c>
+      <c r="D124" t="n">
+        <v>1438</v>
+      </c>
+      <c r="E124" t="n">
+        <v>1895</v>
+      </c>
+      <c r="F124" t="n">
+        <v>0.11387242690418</v>
+      </c>
+      <c r="G124" t="n">
+        <v>0.049416135881464</v>
+      </c>
+      <c r="H124" t="n">
+        <v>0.0212639313198346</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B125" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C125" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D125" t="n">
+        <v>1438</v>
+      </c>
+      <c r="E125" t="n">
+        <v>1895</v>
+      </c>
+      <c r="F125" t="n">
+        <v>0.126534193707734</v>
+      </c>
+      <c r="G125" t="n">
+        <v>0.05141964127036</v>
+      </c>
+      <c r="H125" t="n">
+        <v>0.0139126589673979</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B126" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C126" t="s">
+        <v>1638</v>
+      </c>
+      <c r="D126" t="n">
+        <v>1438</v>
+      </c>
+      <c r="E126" t="n">
+        <v>1895</v>
+      </c>
+      <c r="F126" t="n">
+        <v>0.121583195095758</v>
+      </c>
+      <c r="G126" t="n">
+        <v>0.0520549823357269</v>
+      </c>
+      <c r="H126" t="n">
+        <v>0.0195676514291153</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B127" t="s">
+        <v>3202</v>
+      </c>
+      <c r="C127" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D127" t="n">
+        <v>1438</v>
+      </c>
+      <c r="E127" t="n">
+        <v>1895</v>
+      </c>
+      <c r="F127" t="n">
+        <v>0.104029105739422</v>
+      </c>
+      <c r="G127" t="n">
+        <v>0.0498872890545239</v>
+      </c>
+      <c r="H127" t="n">
+        <v>0.0371197773737983</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
@@ -54449,6 +58731,22 @@
         <v>3191</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>3206</v>
+      </c>
+      <c r="B19" t="s">
+        <v>3207</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>3208</v>
+      </c>
+      <c r="B20" t="s">
+        <v>3209</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>